<commit_message>
feat(inventory): generate executive Sierra Estates Owners Rent Master and Consolidated Rent Master spreadsheets
</commit_message>
<xml_diff>
--- a/apps/sierra-estates-realty/public/downloads/sierra-estates-owners-buy.xlsx
+++ b/apps/sierra-estates-realty/public/downloads/sierra-estates-owners-buy.xlsx
@@ -532,7 +532,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V2" t="str">
-        <v>2026-09-04T14:50:11.197Z</v>
+        <v>2026-09-07T03:58:05.393Z</v>
       </c>
     </row>
     <row r="3">
@@ -1144,7 +1144,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V11" t="str">
-        <v>2026-09-04T14:50:11.197Z</v>
+        <v>2026-09-07T03:58:05.393Z</v>
       </c>
     </row>
     <row r="12" xml:space="preserve">
@@ -1221,7 +1221,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V12" t="str">
-        <v>2026-09-04T14:50:11.197Z</v>
+        <v>2026-09-07T03:58:05.393Z</v>
       </c>
     </row>
     <row r="13">
@@ -1289,7 +1289,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V13" t="str">
-        <v>2026-09-04T14:50:11.197Z</v>
+        <v>2026-09-07T03:58:05.393Z</v>
       </c>
     </row>
     <row r="14">
@@ -1697,7 +1697,7 @@
         <v>Dashboard</v>
       </c>
       <c r="V19" t="str">
-        <v>2026-09-04T14:50:11.197Z</v>
+        <v>2026-09-07T03:58:05.393Z</v>
       </c>
     </row>
     <row r="20">
@@ -1765,7 +1765,7 @@
         <v>Dashboard</v>
       </c>
       <c r="V20" t="str">
-        <v>2026-09-04T14:50:11.197Z</v>
+        <v>2026-09-07T03:58:05.393Z</v>
       </c>
     </row>
     <row r="21">
@@ -1833,7 +1833,7 @@
         <v>Dashboard</v>
       </c>
       <c r="V21" t="str">
-        <v>2026-09-04T14:50:11.197Z</v>
+        <v>2026-09-07T03:58:05.393Z</v>
       </c>
     </row>
     <row r="22">
@@ -1901,7 +1901,7 @@
         <v>Dashboard</v>
       </c>
       <c r="V22" t="str">
-        <v>2026-09-04T14:50:11.197Z</v>
+        <v>2026-09-07T03:58:05.393Z</v>
       </c>
     </row>
     <row r="23">
@@ -2173,7 +2173,7 @@
         <v>Dashboard</v>
       </c>
       <c r="V26" t="str">
-        <v>2026-09-04T14:50:11.197Z</v>
+        <v>2026-09-07T03:58:05.393Z</v>
       </c>
     </row>
     <row r="27">
@@ -2241,7 +2241,7 @@
         <v>Dashboard</v>
       </c>
       <c r="V27" t="str">
-        <v>2026-09-04T14:50:11.197Z</v>
+        <v>2026-09-07T03:58:05.393Z</v>
       </c>
     </row>
     <row r="28">
@@ -2309,7 +2309,7 @@
         <v>Dashboard</v>
       </c>
       <c r="V28" t="str">
-        <v>2026-09-04T14:50:11.197Z</v>
+        <v>2026-09-07T03:58:05.393Z</v>
       </c>
     </row>
     <row r="29" xml:space="preserve">
@@ -2416,7 +2416,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V29" t="str">
-        <v>2026-09-04T14:50:11.197Z</v>
+        <v>2026-09-07T03:58:05.393Z</v>
       </c>
     </row>
     <row r="30">
@@ -2824,7 +2824,7 @@
         <v>Dashboard</v>
       </c>
       <c r="V35" t="str">
-        <v>2026-09-04T14:50:11.197Z</v>
+        <v>2026-09-07T03:58:05.393Z</v>
       </c>
     </row>
     <row r="36">
@@ -3096,7 +3096,7 @@
         <v>Dashboard</v>
       </c>
       <c r="V39" t="str">
-        <v>2026-09-04T14:50:11.197Z</v>
+        <v>2026-09-07T03:58:05.393Z</v>
       </c>
     </row>
     <row r="40">
@@ -3776,7 +3776,7 @@
         <v>Dashboard</v>
       </c>
       <c r="V49" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.393Z</v>
       </c>
     </row>
     <row r="50">
@@ -4184,7 +4184,7 @@
         <v>Dashboard</v>
       </c>
       <c r="V55" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.393Z</v>
       </c>
     </row>
     <row r="56">
@@ -4592,7 +4592,7 @@
         <v>Master Inventory 2026</v>
       </c>
       <c r="V61" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.393Z</v>
       </c>
     </row>
     <row r="62">
@@ -6088,7 +6088,7 @@
         <v>Dashboard</v>
       </c>
       <c r="V83" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.393Z</v>
       </c>
     </row>
     <row r="84">
@@ -6496,7 +6496,7 @@
         <v>Dashboard</v>
       </c>
       <c r="V89" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.393Z</v>
       </c>
     </row>
     <row r="90">
@@ -6564,7 +6564,7 @@
         <v>Dashboard</v>
       </c>
       <c r="V90" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="91">
@@ -6632,7 +6632,7 @@
         <v>Dashboard</v>
       </c>
       <c r="V91" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="92" xml:space="preserve">
@@ -6708,7 +6708,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V92" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="93" xml:space="preserve">
@@ -6793,7 +6793,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V93" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="94">
@@ -6861,7 +6861,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V94" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="95">
@@ -6929,7 +6929,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V95" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="96">
@@ -6997,7 +6997,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V96" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="97">
@@ -7065,7 +7065,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V97" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="98">
@@ -7133,7 +7133,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V98" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="99">
@@ -7201,7 +7201,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V99" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="100">
@@ -7269,7 +7269,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V100" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="101" xml:space="preserve">
@@ -7346,7 +7346,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V101" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="102">
@@ -7414,7 +7414,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V102" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="103">
@@ -7482,7 +7482,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V103" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="104" xml:space="preserve">
@@ -7552,7 +7552,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V104" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="105">
@@ -7620,7 +7620,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V105" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="106" xml:space="preserve">
@@ -7694,7 +7694,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V106" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="107">
@@ -7762,7 +7762,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V107" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="108" xml:space="preserve">
@@ -7843,7 +7843,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V108" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="109" xml:space="preserve">
@@ -7915,7 +7915,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V109" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="110">
@@ -7983,7 +7983,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V110" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="111" xml:space="preserve">
@@ -8061,7 +8061,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V111" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="112">
@@ -8129,7 +8129,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V112" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="113">
@@ -8197,7 +8197,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V113" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="114">
@@ -8265,7 +8265,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V114" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="115">
@@ -8333,7 +8333,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V115" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="116">
@@ -8401,7 +8401,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V116" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="117">
@@ -8469,7 +8469,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V117" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="118">
@@ -8537,7 +8537,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V118" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="119" xml:space="preserve">
@@ -8606,7 +8606,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V119" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="120">
@@ -8674,7 +8674,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V120" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="121">
@@ -8742,7 +8742,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V121" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="122">
@@ -8810,7 +8810,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V122" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="123" xml:space="preserve">
@@ -8889,7 +8889,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V123" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="124">
@@ -8957,7 +8957,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V124" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="125">
@@ -9025,7 +9025,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V125" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="126" xml:space="preserve">
@@ -9179,7 +9179,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V127" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="128">
@@ -9247,7 +9247,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V128" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="129">
@@ -9315,7 +9315,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V129" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="130">
@@ -9383,7 +9383,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V130" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="131">
@@ -9451,7 +9451,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V131" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="132">
@@ -9519,7 +9519,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V132" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="133">
@@ -9587,7 +9587,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V133" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="134">
@@ -9655,7 +9655,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V134" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="135">
@@ -9723,7 +9723,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V135" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="136">
@@ -9791,7 +9791,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V136" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="137">
@@ -9859,7 +9859,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V137" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="138">
@@ -9927,7 +9927,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V138" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="139">
@@ -9995,7 +9995,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V139" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="140">
@@ -10063,7 +10063,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V140" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="141">
@@ -10131,7 +10131,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V141" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="142">
@@ -10199,7 +10199,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V142" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="143">
@@ -10267,7 +10267,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V143" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="144">
@@ -10335,7 +10335,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V144" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="145">
@@ -10403,7 +10403,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V145" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="146">
@@ -10471,7 +10471,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V146" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="147">
@@ -10539,7 +10539,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V147" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="148">
@@ -10607,7 +10607,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V148" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="149">
@@ -10675,7 +10675,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V149" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="150">
@@ -10743,7 +10743,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V150" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="151">
@@ -10811,7 +10811,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V151" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="152">
@@ -10879,7 +10879,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V152" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="153">
@@ -10947,7 +10947,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V153" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="154">
@@ -11015,7 +11015,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V154" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="155">
@@ -11083,7 +11083,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V155" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="156">
@@ -11151,7 +11151,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V156" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="157">
@@ -11219,7 +11219,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V157" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="158">
@@ -11287,7 +11287,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V158" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="159">
@@ -11355,7 +11355,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V159" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="160">
@@ -11423,7 +11423,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V160" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="161">
@@ -11491,7 +11491,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V161" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="162" xml:space="preserve">
@@ -11566,7 +11566,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V162" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="163">
@@ -11634,7 +11634,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V163" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="164">
@@ -11702,7 +11702,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V164" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="165">
@@ -11770,7 +11770,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V165" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="166">
@@ -11838,7 +11838,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V166" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="167">
@@ -11906,7 +11906,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V167" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="168">
@@ -11974,7 +11974,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V168" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="169">
@@ -12042,7 +12042,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V169" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="170" xml:space="preserve">
@@ -12116,7 +12116,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V170" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="171">
@@ -12184,7 +12184,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V171" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="172">
@@ -12320,7 +12320,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V173" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="174">
@@ -12388,7 +12388,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V174" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="175">
@@ -12456,7 +12456,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V175" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="176">
@@ -12524,7 +12524,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V176" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="177">
@@ -12592,7 +12592,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V177" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="178">
@@ -12660,7 +12660,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V178" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="179">
@@ -12728,7 +12728,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V179" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="180">
@@ -12796,7 +12796,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V180" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="181" xml:space="preserve">
@@ -12873,7 +12873,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V181" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="182" xml:space="preserve">
@@ -12949,7 +12949,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V182" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="183" xml:space="preserve">
@@ -13794,7 +13794,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V194" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="195">
@@ -13998,7 +13998,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V197" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="198">
@@ -14066,7 +14066,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V198" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="199">
@@ -14134,7 +14134,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V199" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="200">
@@ -14202,7 +14202,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V200" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="201">
@@ -14270,7 +14270,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V201" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="202">
@@ -14338,7 +14338,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V202" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="203">
@@ -14406,7 +14406,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V203" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="204">
@@ -14542,7 +14542,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V205" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="206">
@@ -14610,7 +14610,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V206" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="207">
@@ -14678,7 +14678,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V207" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="208">
@@ -14746,7 +14746,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V208" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="209">
@@ -14814,7 +14814,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V209" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="210">
@@ -14882,7 +14882,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V210" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="211" xml:space="preserve">
@@ -14955,7 +14955,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V211" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="212">
@@ -15023,7 +15023,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V212" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="213">
@@ -15091,7 +15091,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V213" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="214">
@@ -15227,7 +15227,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V215" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="216" xml:space="preserve">
@@ -15298,7 +15298,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V216" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="217">
@@ -15366,7 +15366,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V217" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="218">
@@ -15434,7 +15434,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V218" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="219" xml:space="preserve">
@@ -15508,7 +15508,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V219" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="220">
@@ -15576,7 +15576,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V220" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="221" xml:space="preserve">
@@ -15651,7 +15651,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V221" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="222">
@@ -15719,7 +15719,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V222" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="223">
@@ -16311,7 +16311,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V230" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="231">
@@ -16379,7 +16379,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V231" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="232">
@@ -16447,7 +16447,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V232" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="233">
@@ -16515,7 +16515,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V233" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="234">
@@ -16583,7 +16583,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V234" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="235">
@@ -16651,7 +16651,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V235" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="236">
@@ -16719,7 +16719,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V236" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="237">
@@ -16787,7 +16787,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V237" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="238">
@@ -16855,7 +16855,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V238" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="239">
@@ -16923,7 +16923,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V239" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="240">
@@ -16991,7 +16991,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V240" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="241">
@@ -17059,7 +17059,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V241" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="242">
@@ -17127,7 +17127,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V242" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="243">
@@ -17195,7 +17195,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V243" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="244">
@@ -17263,7 +17263,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V244" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="245">
@@ -17331,7 +17331,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V245" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="246">
@@ -17399,7 +17399,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V246" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="247">
@@ -17467,7 +17467,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V247" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="248">
@@ -17535,7 +17535,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V248" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="249">
@@ -17603,7 +17603,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V249" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="250">
@@ -17671,7 +17671,7 @@
         <v xml:space="preserve">Owners-Resale </v>
       </c>
       <c r="V250" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="251">
@@ -17739,7 +17739,7 @@
         <v>Master Inventory 2026</v>
       </c>
       <c r="V251" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="252">
@@ -17807,7 +17807,7 @@
         <v>Master Inventory 2026</v>
       </c>
       <c r="V252" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="253">
@@ -17875,7 +17875,7 @@
         <v>Master Inventory 2026</v>
       </c>
       <c r="V253" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="254">
@@ -17943,7 +17943,7 @@
         <v>Master Inventory 2026</v>
       </c>
       <c r="V254" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="255">
@@ -18011,7 +18011,7 @@
         <v>Master Inventory 2026</v>
       </c>
       <c r="V255" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="256">
@@ -18079,7 +18079,7 @@
         <v>Master Inventory 2026</v>
       </c>
       <c r="V256" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="257">
@@ -18215,7 +18215,7 @@
         <v>Dashboard</v>
       </c>
       <c r="V258" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="259">
@@ -18283,7 +18283,7 @@
         <v>Dashboard</v>
       </c>
       <c r="V259" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="260">
@@ -18420,7 +18420,7 @@
         <v>Direct owner</v>
       </c>
       <c r="V261" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="262" xml:space="preserve">
@@ -18489,7 +18489,7 @@
         <v>Direct owner</v>
       </c>
       <c r="V262" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
     <row r="263">
@@ -18557,7 +18557,7 @@
         <v>Direct owner</v>
       </c>
       <c r="V263" t="str">
-        <v>2026-09-04T14:50:11.198Z</v>
+        <v>2026-09-07T03:58:05.394Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>